<commit_message>
Videos for experiments C4-C6, H4-H6
</commit_message>
<xml_diff>
--- a/Code/Tractor Beam/output/Experiment List.xlsx
+++ b/Code/Tractor Beam/output/Experiment List.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\charl\OneDrive\Documents\Projects\Omnimagnet\Code\Tractor Beam\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{416F4502-7679-4686-B49F-B7EE9F526161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7475132D-8552-4348-A728-A4396344BF6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="31">
+  <futureMetadata name="XLRICHVALUE" count="37">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -259,8 +259,50 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="31"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="32"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="33"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="34"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="35"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="36"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="31">
+  <valueMetadata count="37">
     <bk>
       <rc t="1" v="0"/>
     </bk>
@@ -353,13 +395,31 @@
     </bk>
     <bk>
       <rc t="1" v="30"/>
+    </bk>
+    <bk>
+      <rc t="1" v="31"/>
+    </bk>
+    <bk>
+      <rc t="1" v="32"/>
+    </bk>
+    <bk>
+      <rc t="1" v="33"/>
+    </bk>
+    <bk>
+      <rc t="1" v="34"/>
+    </bk>
+    <bk>
+      <rc t="1" v="35"/>
+    </bk>
+    <bk>
+      <rc t="1" v="36"/>
     </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="97">
   <si>
     <t>Experiment</t>
   </si>
@@ -634,13 +694,37 @@
   </si>
   <si>
     <t>Middle raft collides into front and both get pulled in faster than the back raft.</t>
+  </si>
+  <si>
+    <t>Both rafts drift in at similar speeds with the larger raft slightly faster, especially at the end</t>
+  </si>
+  <si>
+    <t>Video 6 Description</t>
+  </si>
+  <si>
+    <t>Video 6 Image</t>
+  </si>
+  <si>
+    <t>Both rafts drift in, large raft drifts faster and catches up to and collides with smaller raft.</t>
+  </si>
+  <si>
+    <t>Both rafts drift in. Large raft has a slow start but ends fast. Small raft has quicker start but maybe lower top speed.</t>
+  </si>
+  <si>
+    <t>Smaller raft catches up to and collides with larger raft the both get pulled in</t>
+  </si>
+  <si>
+    <t>Small raft catches up and collides with larger raft and goes a little past, then larger raft slingshots past</t>
+  </si>
+  <si>
+    <t>Smaller raft catches up to larger raft and both drift in together</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -667,6 +751,12 @@
     <font>
       <sz val="18"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -716,7 +806,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -751,11 +841,26 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="22">
+  <dxfs count="24">
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -764,13 +869,7 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -976,7 +1075,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="31">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="37">
   <rv s="0">
     <v>0</v>
     <v>5</v>
@@ -1099,6 +1198,30 @@
   </rv>
   <rv s="0">
     <v>30</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>31</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>32</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>33</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>34</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>35</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>36</v>
     <v>5</v>
   </rv>
 </rvData>
@@ -1146,32 +1269,40 @@
   <rel r:id="rId29"/>
   <rel r:id="rId30"/>
   <rel r:id="rId31"/>
+  <rel r:id="rId32"/>
+  <rel r:id="rId33"/>
+  <rel r:id="rId34"/>
+  <rel r:id="rId35"/>
+  <rel r:id="rId36"/>
+  <rel r:id="rId37"/>
 </richValueRels>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EFBABB81-F512-4DBE-8388-A4335625DAAC}" name="ExperimentTable" displayName="ExperimentTable" ref="A1:S200" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
-  <autoFilter ref="A1:S200" xr:uid="{EFBABB81-F512-4DBE-8388-A4335625DAAC}"/>
-  <tableColumns count="19">
-    <tableColumn id="1" xr3:uid="{4DD7D756-79AC-47EF-9C53-25636B1735E5}" name="Experiment" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{A5508EBB-85DA-455E-A1FA-9E56CBEDB2BC}" name="Experiment Category" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{EDC4A070-C179-4879-9161-0E6CEE3B03CE}" name="Experiment Variation" dataDxfId="17"/>
-    <tableColumn id="18" xr3:uid="{29A16266-4960-4FC1-9E77-B1F193F89510}" name="Materials Included" dataDxfId="16"/>
-    <tableColumn id="19" xr3:uid="{391AE230-BEFE-47D0-B901-B18AD8DA3BAD}" name="Experiment Group" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{07EC9780-17F5-4E52-B720-72C36789D114}" name="Objects Included" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{E3D8272A-32FA-46B4-9CED-819AE69A7AFC}" name="Layout Photo" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{03820AD5-F5CC-48D3-A203-36988C3D0FE2}" name="Detailed Description" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{4E9FB0B1-757E-473D-A861-553A2A29B87E}" name="Raft Diameters" dataDxfId="11"/>
-    <tableColumn id="8" xr3:uid="{332FF9F0-17E8-45B7-B0F2-B09318E62092}" name="Video 1 Image" dataDxfId="10"/>
-    <tableColumn id="9" xr3:uid="{94CD7315-5538-435F-83A9-A4CC877D8039}" name="Video 1 Description" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{6E20D435-E90D-4EFA-9D84-1818E4341414}" name="Video 2 Image " dataDxfId="8"/>
-    <tableColumn id="11" xr3:uid="{5CFF4F8D-912F-46F5-B8B4-BD7928214C8F}" name="Video 2 Description" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{D5353BFF-361F-44D5-A6B3-B447B5753E0B}" name="Video 3 Image" dataDxfId="6"/>
-    <tableColumn id="13" xr3:uid="{48E41B14-A242-44C3-A9AE-9B7341E870C1}" name="Video 3 Description" dataDxfId="5"/>
-    <tableColumn id="14" xr3:uid="{951F86DC-1089-4B6A-8332-CFFD9F647F43}" name="Video 4 Image " dataDxfId="4"/>
-    <tableColumn id="15" xr3:uid="{4D8E6062-AA59-4A22-8DF7-99FB720B878C}" name="Video 4 Description" dataDxfId="3"/>
-    <tableColumn id="16" xr3:uid="{C4E2EB3A-F870-4D7F-8469-AB06B6E5EBBD}" name="Video 5 Image " dataDxfId="2"/>
-    <tableColumn id="17" xr3:uid="{080AA4D1-4987-4928-BBC4-0F2C293734F6}" name="Video 5 Description" dataDxfId="1"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EFBABB81-F512-4DBE-8388-A4335625DAAC}" name="ExperimentTable" displayName="ExperimentTable" ref="A1:U200" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="A1:U200" xr:uid="{EFBABB81-F512-4DBE-8388-A4335625DAAC}"/>
+  <tableColumns count="21">
+    <tableColumn id="1" xr3:uid="{4DD7D756-79AC-47EF-9C53-25636B1735E5}" name="Experiment" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{A5508EBB-85DA-455E-A1FA-9E56CBEDB2BC}" name="Experiment Category" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{EDC4A070-C179-4879-9161-0E6CEE3B03CE}" name="Experiment Variation" dataDxfId="19"/>
+    <tableColumn id="18" xr3:uid="{29A16266-4960-4FC1-9E77-B1F193F89510}" name="Materials Included" dataDxfId="18"/>
+    <tableColumn id="19" xr3:uid="{391AE230-BEFE-47D0-B901-B18AD8DA3BAD}" name="Experiment Group" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{07EC9780-17F5-4E52-B720-72C36789D114}" name="Objects Included" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{E3D8272A-32FA-46B4-9CED-819AE69A7AFC}" name="Layout Photo" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{03820AD5-F5CC-48D3-A203-36988C3D0FE2}" name="Detailed Description" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{4E9FB0B1-757E-473D-A861-553A2A29B87E}" name="Raft Diameters" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{332FF9F0-17E8-45B7-B0F2-B09318E62092}" name="Video 1 Image" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{94CD7315-5538-435F-83A9-A4CC877D8039}" name="Video 1 Description" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{6E20D435-E90D-4EFA-9D84-1818E4341414}" name="Video 2 Image " dataDxfId="10"/>
+    <tableColumn id="11" xr3:uid="{5CFF4F8D-912F-46F5-B8B4-BD7928214C8F}" name="Video 2 Description" dataDxfId="9"/>
+    <tableColumn id="12" xr3:uid="{D5353BFF-361F-44D5-A6B3-B447B5753E0B}" name="Video 3 Image" dataDxfId="8"/>
+    <tableColumn id="13" xr3:uid="{48E41B14-A242-44C3-A9AE-9B7341E870C1}" name="Video 3 Description" dataDxfId="7"/>
+    <tableColumn id="14" xr3:uid="{951F86DC-1089-4B6A-8332-CFFD9F647F43}" name="Video 4 Image " dataDxfId="6"/>
+    <tableColumn id="15" xr3:uid="{4D8E6062-AA59-4A22-8DF7-99FB720B878C}" name="Video 4 Description" dataDxfId="5"/>
+    <tableColumn id="16" xr3:uid="{C4E2EB3A-F870-4D7F-8469-AB06B6E5EBBD}" name="Video 5 Image " dataDxfId="3"/>
+    <tableColumn id="20" xr3:uid="{98E5A311-33B9-40CC-8CC8-C6461196CB41}" name="Video 5 Description" dataDxfId="2"/>
+    <tableColumn id="21" xr3:uid="{076539AC-1821-45E1-8D80-1E49D0D0C780}" name="Video 6 Image" dataDxfId="1"/>
+    <tableColumn id="17" xr3:uid="{080AA4D1-4987-4928-BBC4-0F2C293734F6}" name="Video 6 Description" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium13" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1440,7 +1571,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S12"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="17.3125" style="5" customWidth="1"/>
@@ -1458,14 +1589,16 @@
     <col min="14" max="14" width="37.7890625" style="2" customWidth="1"/>
     <col min="15" max="15" width="27.41796875" style="7" customWidth="1"/>
     <col min="16" max="16" width="37.83984375" style="2" customWidth="1"/>
-    <col min="17" max="17" width="27.41796875" style="2" customWidth="1"/>
+    <col min="17" max="17" width="27.41796875" style="7" customWidth="1"/>
     <col min="18" max="18" width="37.9453125" style="2" customWidth="1"/>
-    <col min="19" max="19" width="27.41796875" style="2" customWidth="1"/>
-    <col min="20" max="25" width="27.41796875" style="2" hidden="1" customWidth="1"/>
-    <col min="26" max="16384" width="27.41796875" style="2" hidden="1"/>
+    <col min="19" max="19" width="37.9453125" style="7" customWidth="1"/>
+    <col min="20" max="20" width="37.9453125" style="2" customWidth="1"/>
+    <col min="21" max="21" width="38.26171875" style="7" customWidth="1"/>
+    <col min="22" max="27" width="27.41796875" style="2" hidden="1" customWidth="1"/>
+    <col min="28" max="16384" width="27.41796875" style="2" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="4" customFormat="1" ht="63.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:21" s="4" customFormat="1" ht="63.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1514,7 +1647,7 @@
       <c r="P1" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="Q1" s="12" t="s">
         <v>50</v>
       </c>
       <c r="R1" s="4" t="s">
@@ -1523,8 +1656,14 @@
       <c r="S1" s="4" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="2" spans="1:19" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="T1" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="U1" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -1571,7 +1710,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:21" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
@@ -1618,7 +1757,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:21" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="5" t="s">
         <v>3</v>
       </c>
@@ -1664,8 +1803,26 @@
       <c r="O4" s="11" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="5" spans="1:19" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="P4" s="2" t="e" vm="13">
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q4" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="R4" s="2" t="e" vm="14">
+        <v>#VALUE!</v>
+      </c>
+      <c r="S4" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="T4" s="2" t="e" vm="15">
+        <v>#VALUE!</v>
+      </c>
+      <c r="U4" s="7" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
@@ -1684,7 +1841,7 @@
       <c r="F5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="3" t="e" vm="13">
+      <c r="G5" s="3" t="e" vm="16">
         <v>#VALUE!</v>
       </c>
       <c r="H5" s="7" t="s">
@@ -1693,26 +1850,26 @@
       <c r="I5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J5" s="1" t="e" vm="14">
+      <c r="J5" s="1" t="e" vm="17">
         <v>#VALUE!</v>
       </c>
       <c r="K5" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="L5" s="1" t="e" vm="15">
+      <c r="L5" s="1" t="e" vm="18">
         <v>#VALUE!</v>
       </c>
       <c r="M5" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="N5" s="2" t="e" vm="16">
+      <c r="N5" s="2" t="e" vm="19">
         <v>#VALUE!</v>
       </c>
       <c r="O5" s="9" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:21" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="5" t="s">
         <v>13</v>
       </c>
@@ -1731,7 +1888,7 @@
       <c r="F6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="3" t="e" vm="17">
+      <c r="G6" s="3" t="e" vm="20">
         <v>#VALUE!</v>
       </c>
       <c r="H6" s="7" t="s">
@@ -1740,26 +1897,26 @@
       <c r="I6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J6" s="1" t="e" vm="18">
+      <c r="J6" s="1" t="e" vm="21">
         <v>#VALUE!</v>
       </c>
       <c r="K6" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="L6" s="1" t="e" vm="18">
+      <c r="L6" s="1" t="e" vm="21">
         <v>#VALUE!</v>
       </c>
       <c r="M6" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="N6" s="2" t="e" vm="19">
+      <c r="N6" s="2" t="e" vm="22">
         <v>#VALUE!</v>
       </c>
       <c r="O6" s="11" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:21" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="5" t="s">
         <v>17</v>
       </c>
@@ -1778,7 +1935,7 @@
       <c r="F7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="3" t="e" vm="20">
+      <c r="G7" s="3" t="e" vm="23">
         <v>#VALUE!</v>
       </c>
       <c r="H7" s="7" t="s">
@@ -1787,26 +1944,26 @@
       <c r="I7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J7" s="1" t="e" vm="21">
+      <c r="J7" s="1" t="e" vm="24">
         <v>#VALUE!</v>
       </c>
       <c r="K7" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="L7" s="1" t="e" vm="22">
+      <c r="L7" s="1" t="e" vm="25">
         <v>#VALUE!</v>
       </c>
       <c r="M7" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="N7" s="2" t="e" vm="23">
+      <c r="N7" s="2" t="e" vm="26">
         <v>#VALUE!</v>
       </c>
       <c r="O7" s="10" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:21" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="5" t="s">
         <v>19</v>
       </c>
@@ -1825,7 +1982,7 @@
       <c r="F8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="3" t="e" vm="24">
+      <c r="G8" s="3" t="e" vm="27">
         <v>#VALUE!</v>
       </c>
       <c r="H8" s="7" t="s">
@@ -1834,26 +1991,26 @@
       <c r="I8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J8" s="1" t="e" vm="25">
+      <c r="J8" s="1" t="e" vm="28">
         <v>#VALUE!</v>
       </c>
       <c r="K8" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="L8" s="1" t="e" vm="26">
+      <c r="L8" s="1" t="e" vm="29">
         <v>#VALUE!</v>
       </c>
       <c r="M8" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="N8" s="2" t="e" vm="27">
+      <c r="N8" s="2" t="e" vm="30">
         <v>#VALUE!</v>
       </c>
       <c r="O8" s="11" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:21" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="5" t="s">
         <v>58</v>
       </c>
@@ -1872,7 +2029,7 @@
       <c r="F9" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="G9" s="3" t="e" vm="28">
+      <c r="G9" s="3" t="e" vm="31">
         <v>#VALUE!</v>
       </c>
       <c r="H9" s="7" t="s">
@@ -1881,26 +2038,44 @@
       <c r="I9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J9" s="1" t="e" vm="29">
+      <c r="J9" s="1" t="e" vm="32">
         <v>#VALUE!</v>
       </c>
       <c r="K9" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="L9" s="1" t="e" vm="30">
+      <c r="L9" s="1" t="e" vm="33">
         <v>#VALUE!</v>
       </c>
       <c r="M9" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="N9" s="2" t="e" vm="31">
+      <c r="N9" s="2" t="e" vm="34">
         <v>#VALUE!</v>
       </c>
       <c r="O9" s="10" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="10" spans="1:19" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="P9" s="2" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="R9" s="2" t="e" vm="36">
+        <v>#VALUE!</v>
+      </c>
+      <c r="S9" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="T9" s="2" t="e" vm="37">
+        <v>#VALUE!</v>
+      </c>
+      <c r="U9" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="5" t="s">
         <v>65</v>
       </c>
@@ -1926,7 +2101,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:21" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="5" t="s">
         <v>66</v>
       </c>
@@ -1952,7 +2127,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:21" ht="112.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="5" t="s">
         <v>67</v>
       </c>
@@ -1979,8 +2154,9 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="J1:S200">
-    <cfRule type="expression" dxfId="0" priority="1">
+  <phoneticPr fontId="4" type="noConversion"/>
+  <conditionalFormatting sqref="J1:U200">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>ISBLANK(J1)</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>